<commit_message>
Sync SYAVLo and AVLo values
</commit_message>
<xml_diff>
--- a/InputData/trans/AVLo/Avg Vehicle Loading.xlsx
+++ b/InputData/trans/AVLo/Avg Vehicle Loading.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\DanOBrien\Models\EPS\SK\eps-southkorea\InputData\trans\AVLo\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Mary Francis Swint\Vensim\eps-southkorea\InputData\trans\AVLo\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{DFE894FA-EC83-4559-89EE-D4C2A33FC530}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{42A4C623-08CD-46A8-883B-486664EAAE22}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{93120D57-562B-4CC7-BC2A-853A917AD7F3}"/>
+    <workbookView xWindow="-38505" yWindow="-2205" windowWidth="19410" windowHeight="20985" firstSheet="12" activeTab="13" xr2:uid="{93120D57-562B-4CC7-BC2A-853A917AD7F3}"/>
   </bookViews>
   <sheets>
     <sheet name="About" sheetId="1" r:id="rId1"/>
@@ -4386,13 +4386,35 @@
 </a:theme>
 </file>
 
+<file path=xl/webextensions/taskpanes.xml><?xml version="1.0" encoding="utf-8"?>
+<wetp:taskpanes xmlns:wetp="http://schemas.microsoft.com/office/webextensions/taskpanes/2010/11">
+  <wetp:taskpane dockstate="right" visibility="0" width="350" row="7">
+    <wetp:webextensionref xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+  </wetp:taskpane>
+</wetp:taskpanes>
+</file>
+
+<file path=xl/webextensions/webextension1.xml><?xml version="1.0" encoding="utf-8"?>
+<we:webextension xmlns:we="http://schemas.microsoft.com/office/webextensions/webextension/2010/11" id="{CB97A2CC-A3B7-4442-973C-5AD563F0CA49}">
+  <we:reference id="WA200009404" version="1.0.0.8" store="Omex" storeType="OMEX"/>
+  <we:alternateReferences>
+    <we:reference id="WA200009404" version="1.0.0.8" store="WA200009404" storeType="OMEX"/>
+  </we:alternateReferences>
+  <we:properties>
+    <we:property name="claude.fileId" value="&quot;d5141e47-7ec8-423e-90d9-571e7acd7f4f&quot;"/>
+  </we:properties>
+  <we:bindings/>
+  <we:snapshot xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships"/>
+</we:webextension>
+</file>
+
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:F42"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="11.42578125" customWidth="1"/>
-    <col min="2" max="2" width="85.140625" customWidth="1"/>
+    <col min="1" max="1" width="11.453125" customWidth="1"/>
+    <col min="2" max="2" width="85.1796875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6">
@@ -4639,13 +4661,13 @@
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{39261612-B7A0-4B40-8A97-686A4FA3FEBF}">
   <dimension ref="A1:M60"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="2" width="10.85546875" customWidth="1"/>
-    <col min="3" max="3" width="13.42578125" customWidth="1"/>
-    <col min="4" max="7" width="10.85546875" customWidth="1"/>
-    <col min="10" max="10" width="15.42578125" customWidth="1"/>
-    <col min="11" max="11" width="14.42578125" customWidth="1"/>
+    <col min="1" max="2" width="10.81640625" customWidth="1"/>
+    <col min="3" max="3" width="13.453125" customWidth="1"/>
+    <col min="4" max="7" width="10.81640625" customWidth="1"/>
+    <col min="10" max="10" width="15.453125" customWidth="1"/>
+    <col min="11" max="11" width="14.453125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:1">
@@ -4756,7 +4778,7 @@
         <v>338</v>
       </c>
     </row>
-    <row r="38" spans="1:13" ht="45">
+    <row r="38" spans="1:13" ht="43.5">
       <c r="A38" s="110" t="s">
         <v>329</v>
       </c>
@@ -5216,7 +5238,7 @@
         <v>330</v>
       </c>
     </row>
-    <row r="54" spans="1:13" ht="30">
+    <row r="54" spans="1:13" ht="29">
       <c r="A54" s="110" t="s">
         <v>329</v>
       </c>
@@ -5348,13 +5370,13 @@
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9438158E-C803-4774-ADE5-31C8503BC4B7}">
   <dimension ref="A1:Q31"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="2" max="3" width="14.85546875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="8.85546875" customWidth="1"/>
+    <col min="2" max="3" width="14.81640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="8.81640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" ht="15.75" thickBot="1">
+    <row r="1" spans="1:9" ht="15" thickBot="1">
       <c r="A1" s="27" t="s">
         <v>171</v>
       </c>
@@ -5378,7 +5400,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="3" spans="1:9" ht="15.75" thickBot="1">
+    <row r="3" spans="1:9" ht="15" thickBot="1">
       <c r="A3" s="90"/>
       <c r="B3" s="72"/>
       <c r="C3" s="137" t="s">
@@ -5394,7 +5416,7 @@
       <c r="G3" s="72"/>
       <c r="H3" s="73"/>
     </row>
-    <row r="4" spans="1:9" ht="15.75" thickTop="1">
+    <row r="4" spans="1:9" ht="15" thickTop="1">
       <c r="A4" s="87" t="s">
         <v>210</v>
       </c>
@@ -5457,7 +5479,7 @@
         <v>112</v>
       </c>
     </row>
-    <row r="7" spans="1:9" ht="15.75" thickBot="1">
+    <row r="7" spans="1:9" ht="15" thickBot="1">
       <c r="A7" s="90"/>
       <c r="B7" s="91"/>
       <c r="C7" s="91"/>
@@ -5470,7 +5492,7 @@
       <c r="H7" s="92"/>
       <c r="I7" s="32"/>
     </row>
-    <row r="8" spans="1:9" ht="15.75" thickTop="1">
+    <row r="8" spans="1:9" ht="15" thickTop="1">
       <c r="A8" s="87" t="s">
         <v>209</v>
       </c>
@@ -5494,7 +5516,7 @@
         <v>263</v>
       </c>
     </row>
-    <row r="9" spans="1:9" ht="15.75" thickBot="1">
+    <row r="9" spans="1:9" ht="15" thickBot="1">
       <c r="A9" s="69"/>
       <c r="B9" s="89" t="s">
         <v>212</v>
@@ -5520,7 +5542,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="11" spans="1:9" ht="17.25">
+    <row r="11" spans="1:9" ht="17.5">
       <c r="B11" s="63" t="s">
         <v>207</v>
       </c>
@@ -5596,7 +5618,7 @@
         <v>206</v>
       </c>
     </row>
-    <row r="28" spans="1:17" ht="15.75" thickBot="1">
+    <row r="28" spans="1:17" ht="15" thickBot="1">
       <c r="A28" s="7" t="s">
         <v>115</v>
       </c>
@@ -5605,7 +5627,7 @@
       <c r="D28" s="8"/>
       <c r="H28" s="1"/>
     </row>
-    <row r="29" spans="1:17" ht="15.75" thickBot="1">
+    <row r="29" spans="1:17" ht="15" thickBot="1">
       <c r="A29" s="80"/>
       <c r="B29" s="81" t="s">
         <v>55</v>
@@ -5620,7 +5642,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="30" spans="1:17" ht="15.75" thickTop="1">
+    <row r="30" spans="1:17" ht="15" thickTop="1">
       <c r="A30" s="77" t="s">
         <v>58</v>
       </c>
@@ -5639,7 +5661,7 @@
         <v>208</v>
       </c>
     </row>
-    <row r="31" spans="1:17" ht="15.75" thickBot="1">
+    <row r="31" spans="1:17" ht="15" thickBot="1">
       <c r="A31" s="74" t="s">
         <v>59</v>
       </c>
@@ -5671,7 +5693,7 @@
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0D8AABE4-9A7A-4FF9-8C38-25844DE09CA8}">
   <dimension ref="A1:AK15"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
   <sheetData>
     <row r="1" spans="1:37">
       <c r="A1" t="s">
@@ -7246,13 +7268,13 @@
     <tabColor theme="3"/>
   </sheetPr>
   <dimension ref="A1:AK7"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="13.140625" customWidth="1"/>
-    <col min="2" max="2" width="8.7109375" customWidth="1"/>
+    <col min="1" max="1" width="13.1796875" customWidth="1"/>
+    <col min="2" max="2" width="8.7265625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:37" ht="45">
+    <row r="1" spans="1:37" ht="43.5">
       <c r="A1" s="6" t="s">
         <v>9</v>
       </c>
@@ -7300,8 +7322,8 @@
         <v>2</v>
       </c>
       <c r="B2" s="4">
-        <f>'DV-psgr'!H41*'DV-psgr'!K41</f>
-        <v>1.1232755332153297</v>
+        <f>'AVLo-passengers'!G2</f>
+        <v>1.0530708123893715</v>
       </c>
       <c r="C2" s="4"/>
       <c r="D2" s="4"/>
@@ -7343,8 +7365,8 @@
       <c r="A3" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="B3" s="5">
-        <f>'DV-psgr'!H42</f>
+      <c r="B3" s="4">
+        <f>'AVLo-passengers'!G3</f>
         <v>14.731070293267342</v>
       </c>
       <c r="C3" s="4"/>
@@ -7387,9 +7409,9 @@
       <c r="A4" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B4" s="5">
-        <f>'Air-Calcs'!M47</f>
-        <v>145.95406739643701</v>
+      <c r="B4" s="4">
+        <f>'AVLo-passengers'!G4</f>
+        <v>155.72981935122084</v>
       </c>
       <c r="C4" s="4"/>
       <c r="D4" s="4"/>
@@ -7431,8 +7453,8 @@
       <c r="A5" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="B5" s="5">
-        <f>rail!D30</f>
+      <c r="B5" s="4">
+        <f>'AVLo-passengers'!G5</f>
         <v>382.85954795395736</v>
       </c>
       <c r="C5" s="4"/>
@@ -7476,7 +7498,7 @@
         <v>6</v>
       </c>
       <c r="B6" s="4">
-        <f>'ships-psgr'!G3</f>
+        <f>'AVLo-passengers'!G6</f>
         <v>337.61417769892506</v>
       </c>
       <c r="C6" s="4"/>
@@ -7519,7 +7541,8 @@
       <c r="A7" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="B7" s="24">
+      <c r="B7" s="4">
+        <f>'AVLo-passengers'!G7</f>
         <v>1.1000000000000001</v>
       </c>
       <c r="C7" s="4"/>
@@ -7570,12 +7593,12 @@
     <tabColor theme="3"/>
   </sheetPr>
   <dimension ref="A1:AJ7"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="11.85546875" customWidth="1"/>
+    <col min="1" max="1" width="11.81640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:36" s="1" customFormat="1" ht="45">
+    <row r="1" spans="1:36" s="1" customFormat="1" ht="43.5">
       <c r="A1" s="6" t="s">
         <v>10</v>
       </c>
@@ -7588,7 +7611,7 @@
         <v>2</v>
       </c>
       <c r="B2" s="125">
-        <f>'DV-freight'!P28</f>
+        <f>'AVLo-freight'!F2</f>
         <v>0.56135536398467423</v>
       </c>
       <c r="C2" s="28"/>
@@ -7631,7 +7654,7 @@
         <v>3</v>
       </c>
       <c r="B3" s="126">
-        <f>'DV-freight'!P31</f>
+        <f>'AVLo-freight'!F3</f>
         <v>6.6919426527303214</v>
       </c>
     </row>
@@ -7640,7 +7663,7 @@
         <v>4</v>
       </c>
       <c r="B4" s="29">
-        <f>BAADTbVT_air!L9</f>
+        <f>'AVLo-freight'!F4</f>
         <v>63.556825639903742</v>
       </c>
       <c r="C4" s="3"/>
@@ -7683,7 +7706,7 @@
         <v>5</v>
       </c>
       <c r="B5" s="29">
-        <f>rail!C15</f>
+        <f>'AVLo-freight'!F5</f>
         <v>1514.4</v>
       </c>
       <c r="C5" s="3"/>
@@ -7726,7 +7749,7 @@
         <v>6</v>
       </c>
       <c r="B6" s="106">
-        <f>'US AVLo'!$B$14</f>
+        <f>'AVLo-freight'!F6</f>
         <v>1974.4736422180429</v>
       </c>
       <c r="C6" s="106"/>
@@ -7769,6 +7792,7 @@
         <v>7</v>
       </c>
       <c r="B7" s="25">
+        <f>'AVLo-freight'!F7</f>
         <v>3.0000000000000001E-3</v>
       </c>
     </row>
@@ -7785,13 +7809,13 @@
     <tabColor theme="3"/>
   </sheetPr>
   <dimension ref="A1:AK7"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="13.140625" customWidth="1"/>
-    <col min="2" max="2" width="8.7109375" customWidth="1"/>
+    <col min="1" max="1" width="13.1796875" customWidth="1"/>
+    <col min="2" max="2" width="8.7265625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:37" ht="45">
+    <row r="1" spans="1:37" ht="43.5">
       <c r="A1" s="6" t="s">
         <v>9</v>
       </c>
@@ -8806,12 +8830,12 @@
     <tabColor theme="3"/>
   </sheetPr>
   <dimension ref="A1:AJ7"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="11.85546875" customWidth="1"/>
+    <col min="1" max="1" width="11.81640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:36" s="1" customFormat="1" ht="45">
+    <row r="1" spans="1:36" s="1" customFormat="1" ht="43.5">
       <c r="A1" s="6" t="s">
         <v>10</v>
       </c>
@@ -9800,10 +9824,10 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B6E22F11-BE45-4915-A8C3-90BE8CB5DD1C}">
   <dimension ref="A39:T61"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="3" max="3" width="12.85546875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.85546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.81640625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.81640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="39" spans="2:20">
@@ -10074,15 +10098,15 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AAD3B914-B72F-432B-8D51-3CBE259118E1}">
   <dimension ref="A1:P47"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.5"/>
   <cols>
     <col min="1" max="11" width="9" style="8"/>
-    <col min="12" max="12" width="10.85546875" style="8" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="10.81640625" style="8" bestFit="1" customWidth="1"/>
     <col min="13" max="13" width="9" style="8" customWidth="1"/>
-    <col min="14" max="14" width="16.28515625" style="8" customWidth="1"/>
-    <col min="15" max="15" width="18.42578125" style="8" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="16.26953125" style="8" customWidth="1"/>
+    <col min="15" max="15" width="18.453125" style="8" bestFit="1" customWidth="1"/>
     <col min="16" max="16" width="9" style="8"/>
-    <col min="17" max="17" width="13.42578125" style="8" customWidth="1"/>
+    <col min="17" max="17" width="13.453125" style="8" customWidth="1"/>
     <col min="18" max="16384" width="9" style="8"/>
   </cols>
   <sheetData>
@@ -10925,23 +10949,23 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{152A55CB-ED11-48EF-AA99-B206FDDEB829}">
   <dimension ref="A1:P55"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.5"/>
   <cols>
     <col min="1" max="1" width="10" style="8" customWidth="1"/>
-    <col min="2" max="2" width="13.140625" style="8" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="23.28515625" style="8" customWidth="1"/>
-    <col min="4" max="4" width="13.140625" style="8" customWidth="1"/>
-    <col min="5" max="5" width="23.140625" style="8" customWidth="1"/>
-    <col min="6" max="6" width="9.5703125" style="8" customWidth="1"/>
-    <col min="7" max="7" width="14.28515625" style="8" customWidth="1"/>
-    <col min="8" max="8" width="14.7109375" style="8" customWidth="1"/>
-    <col min="9" max="9" width="15.140625" style="8" customWidth="1"/>
-    <col min="10" max="10" width="12.28515625" style="8" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="15.85546875" style="8" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="9.140625" style="8" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="15.85546875" style="8" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="17.7109375" style="8" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="12.7109375" style="8" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="13.1796875" style="8" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="23.26953125" style="8" customWidth="1"/>
+    <col min="4" max="4" width="13.1796875" style="8" customWidth="1"/>
+    <col min="5" max="5" width="23.1796875" style="8" customWidth="1"/>
+    <col min="6" max="6" width="9.54296875" style="8" customWidth="1"/>
+    <col min="7" max="7" width="14.26953125" style="8" customWidth="1"/>
+    <col min="8" max="8" width="14.7265625" style="8" customWidth="1"/>
+    <col min="9" max="9" width="15.1796875" style="8" customWidth="1"/>
+    <col min="10" max="10" width="12.26953125" style="8" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="15.81640625" style="8" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="9.1796875" style="8" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="15.81640625" style="8" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="17.7265625" style="8" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="12.7265625" style="8" bestFit="1" customWidth="1"/>
     <col min="16" max="16384" width="9" style="8"/>
   </cols>
   <sheetData>
@@ -12594,16 +12618,16 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8DBB0CBB-759C-4C56-A4C4-D4E65F9775FA}">
   <dimension ref="B2:I175"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="2" max="2" width="10.7109375" customWidth="1"/>
-    <col min="5" max="5" width="15.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.7265625" customWidth="1"/>
+    <col min="5" max="5" width="15.81640625" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="19" customWidth="1"/>
-    <col min="7" max="7" width="20.42578125" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="18.42578125" customWidth="1"/>
+    <col min="7" max="7" width="20.453125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="18.453125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:9" ht="15.75" thickBot="1">
+    <row r="2" spans="2:9" ht="15" thickBot="1">
       <c r="B2" s="40" t="s">
         <v>104</v>
       </c>
@@ -12717,7 +12741,7 @@
         <v>254.87619047619049</v>
       </c>
     </row>
-    <row r="8" spans="2:9" ht="15.75" thickBot="1">
+    <row r="8" spans="2:9" ht="15" thickBot="1">
       <c r="B8" s="27" t="s">
         <v>98</v>
       </c>
@@ -12754,7 +12778,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="13" spans="2:9" ht="15.75" thickBot="1">
+    <row r="13" spans="2:9" ht="15" thickBot="1">
       <c r="B13" s="40" t="s">
         <v>104</v>
       </c>
@@ -12904,7 +12928,7 @@
         <v>254.87619047619049</v>
       </c>
     </row>
-    <row r="19" spans="2:9" ht="15.75" thickBot="1">
+    <row r="19" spans="2:9" ht="15" thickBot="1">
       <c r="B19" t="s">
         <v>96</v>
       </c>
@@ -14661,11 +14685,11 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{ACC9CD64-51B3-4C21-ABDF-5DD1D16C3DC4}">
   <dimension ref="A1:H29"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="16.42578125" customWidth="1"/>
-    <col min="3" max="4" width="9.42578125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="15.42578125" customWidth="1"/>
+    <col min="1" max="1" width="16.453125" customWidth="1"/>
+    <col min="3" max="4" width="9.453125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="15.453125" customWidth="1"/>
     <col min="8" max="8" width="9" customWidth="1"/>
   </cols>
   <sheetData>
@@ -14674,7 +14698,7 @@
         <v>274</v>
       </c>
     </row>
-    <row r="2" spans="1:7" ht="15.75" thickBot="1">
+    <row r="2" spans="1:7" ht="15" thickBot="1">
       <c r="A2" s="103" t="s">
         <v>275</v>
       </c>
@@ -15078,7 +15102,7 @@
         <v>45.8</v>
       </c>
     </row>
-    <row r="21" spans="1:8" ht="15.75" thickBot="1">
+    <row r="21" spans="1:8" ht="15" thickBot="1">
       <c r="A21" s="91" t="s">
         <v>297</v>
       </c>
@@ -15096,7 +15120,7 @@
         <v>25406.090909090908</v>
       </c>
     </row>
-    <row r="22" spans="1:8" ht="15.75" thickTop="1">
+    <row r="22" spans="1:8" ht="15" thickTop="1">
       <c r="A22" s="102" t="s">
         <v>53</v>
       </c>
@@ -15130,7 +15154,7 @@
         <v>299</v>
       </c>
     </row>
-    <row r="25" spans="1:8" ht="15.75" thickBot="1">
+    <row r="25" spans="1:8" ht="15" thickBot="1">
       <c r="A25" s="130" t="s">
         <v>300</v>
       </c>
@@ -15267,27 +15291,27 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{834C8993-7EE0-4137-9B77-501005A3F9D6}">
   <dimension ref="A2:N49"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="11.7109375" style="8" customWidth="1"/>
+    <col min="1" max="1" width="11.7265625" style="8" customWidth="1"/>
     <col min="2" max="2" width="9" style="8"/>
-    <col min="3" max="4" width="11.42578125" style="8" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="9.85546875" style="8" bestFit="1" customWidth="1"/>
+    <col min="3" max="4" width="11.453125" style="8" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="9.81640625" style="8" bestFit="1" customWidth="1"/>
     <col min="6" max="7" width="9" style="8"/>
-    <col min="8" max="8" width="8.85546875" style="8" customWidth="1"/>
-    <col min="9" max="9" width="12.42578125" style="8" customWidth="1"/>
-    <col min="10" max="10" width="3.7109375" style="8" customWidth="1"/>
-    <col min="11" max="11" width="4.42578125" style="8" customWidth="1"/>
-    <col min="12" max="12" width="20.28515625" style="8" customWidth="1"/>
+    <col min="8" max="8" width="8.81640625" style="8" customWidth="1"/>
+    <col min="9" max="9" width="12.453125" style="8" customWidth="1"/>
+    <col min="10" max="10" width="3.7265625" style="8" customWidth="1"/>
+    <col min="11" max="11" width="4.453125" style="8" customWidth="1"/>
+    <col min="12" max="12" width="20.26953125" style="8" customWidth="1"/>
     <col min="13" max="13" width="17" style="8" customWidth="1"/>
     <col min="14" max="14" width="18" style="8" customWidth="1"/>
     <col min="15" max="16" width="9" style="8"/>
-    <col min="17" max="17" width="11.140625" style="8" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="18.28515625" style="8" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="11.1796875" style="8" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="18.26953125" style="8" bestFit="1" customWidth="1"/>
     <col min="19" max="16384" width="9" style="8"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:12" ht="15.75" thickBot="1">
+    <row r="2" spans="2:12" ht="15" thickBot="1">
       <c r="D2" s="43" t="s">
         <v>129</v>
       </c>
@@ -15558,7 +15582,7 @@
         <v>43669</v>
       </c>
     </row>
-    <row r="16" spans="2:12" ht="15.75" thickBot="1">
+    <row r="16" spans="2:12" ht="15" thickBot="1">
       <c r="B16" s="49">
         <v>2018</v>
       </c>
@@ -16552,456 +16576,456 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{08F5C122-988D-446F-A1DB-C3D7ACE874B7}">
   <dimension ref="A1:R23"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="21.140625" customWidth="1"/>
-    <col min="2" max="2" width="12.42578125" customWidth="1"/>
-    <col min="3" max="7" width="12.7109375" customWidth="1"/>
-    <col min="8" max="8" width="12.85546875" customWidth="1"/>
-    <col min="9" max="10" width="12.7109375" customWidth="1"/>
-    <col min="11" max="14" width="12.85546875" customWidth="1"/>
-    <col min="15" max="18" width="12.7109375" customWidth="1"/>
-    <col min="257" max="257" width="21.140625" customWidth="1"/>
-    <col min="258" max="258" width="12.42578125" customWidth="1"/>
-    <col min="259" max="263" width="12.7109375" customWidth="1"/>
-    <col min="264" max="264" width="12.85546875" customWidth="1"/>
-    <col min="265" max="266" width="12.7109375" customWidth="1"/>
-    <col min="267" max="270" width="12.85546875" customWidth="1"/>
-    <col min="271" max="274" width="12.7109375" customWidth="1"/>
-    <col min="513" max="513" width="21.140625" customWidth="1"/>
-    <col min="514" max="514" width="12.42578125" customWidth="1"/>
-    <col min="515" max="519" width="12.7109375" customWidth="1"/>
-    <col min="520" max="520" width="12.85546875" customWidth="1"/>
-    <col min="521" max="522" width="12.7109375" customWidth="1"/>
-    <col min="523" max="526" width="12.85546875" customWidth="1"/>
-    <col min="527" max="530" width="12.7109375" customWidth="1"/>
-    <col min="769" max="769" width="21.140625" customWidth="1"/>
-    <col min="770" max="770" width="12.42578125" customWidth="1"/>
-    <col min="771" max="775" width="12.7109375" customWidth="1"/>
-    <col min="776" max="776" width="12.85546875" customWidth="1"/>
-    <col min="777" max="778" width="12.7109375" customWidth="1"/>
-    <col min="779" max="782" width="12.85546875" customWidth="1"/>
-    <col min="783" max="786" width="12.7109375" customWidth="1"/>
-    <col min="1025" max="1025" width="21.140625" customWidth="1"/>
-    <col min="1026" max="1026" width="12.42578125" customWidth="1"/>
-    <col min="1027" max="1031" width="12.7109375" customWidth="1"/>
-    <col min="1032" max="1032" width="12.85546875" customWidth="1"/>
-    <col min="1033" max="1034" width="12.7109375" customWidth="1"/>
-    <col min="1035" max="1038" width="12.85546875" customWidth="1"/>
-    <col min="1039" max="1042" width="12.7109375" customWidth="1"/>
-    <col min="1281" max="1281" width="21.140625" customWidth="1"/>
-    <col min="1282" max="1282" width="12.42578125" customWidth="1"/>
-    <col min="1283" max="1287" width="12.7109375" customWidth="1"/>
-    <col min="1288" max="1288" width="12.85546875" customWidth="1"/>
-    <col min="1289" max="1290" width="12.7109375" customWidth="1"/>
-    <col min="1291" max="1294" width="12.85546875" customWidth="1"/>
-    <col min="1295" max="1298" width="12.7109375" customWidth="1"/>
-    <col min="1537" max="1537" width="21.140625" customWidth="1"/>
-    <col min="1538" max="1538" width="12.42578125" customWidth="1"/>
-    <col min="1539" max="1543" width="12.7109375" customWidth="1"/>
-    <col min="1544" max="1544" width="12.85546875" customWidth="1"/>
-    <col min="1545" max="1546" width="12.7109375" customWidth="1"/>
-    <col min="1547" max="1550" width="12.85546875" customWidth="1"/>
-    <col min="1551" max="1554" width="12.7109375" customWidth="1"/>
-    <col min="1793" max="1793" width="21.140625" customWidth="1"/>
-    <col min="1794" max="1794" width="12.42578125" customWidth="1"/>
-    <col min="1795" max="1799" width="12.7109375" customWidth="1"/>
-    <col min="1800" max="1800" width="12.85546875" customWidth="1"/>
-    <col min="1801" max="1802" width="12.7109375" customWidth="1"/>
-    <col min="1803" max="1806" width="12.85546875" customWidth="1"/>
-    <col min="1807" max="1810" width="12.7109375" customWidth="1"/>
-    <col min="2049" max="2049" width="21.140625" customWidth="1"/>
-    <col min="2050" max="2050" width="12.42578125" customWidth="1"/>
-    <col min="2051" max="2055" width="12.7109375" customWidth="1"/>
-    <col min="2056" max="2056" width="12.85546875" customWidth="1"/>
-    <col min="2057" max="2058" width="12.7109375" customWidth="1"/>
-    <col min="2059" max="2062" width="12.85546875" customWidth="1"/>
-    <col min="2063" max="2066" width="12.7109375" customWidth="1"/>
-    <col min="2305" max="2305" width="21.140625" customWidth="1"/>
-    <col min="2306" max="2306" width="12.42578125" customWidth="1"/>
-    <col min="2307" max="2311" width="12.7109375" customWidth="1"/>
-    <col min="2312" max="2312" width="12.85546875" customWidth="1"/>
-    <col min="2313" max="2314" width="12.7109375" customWidth="1"/>
-    <col min="2315" max="2318" width="12.85546875" customWidth="1"/>
-    <col min="2319" max="2322" width="12.7109375" customWidth="1"/>
-    <col min="2561" max="2561" width="21.140625" customWidth="1"/>
-    <col min="2562" max="2562" width="12.42578125" customWidth="1"/>
-    <col min="2563" max="2567" width="12.7109375" customWidth="1"/>
-    <col min="2568" max="2568" width="12.85546875" customWidth="1"/>
-    <col min="2569" max="2570" width="12.7109375" customWidth="1"/>
-    <col min="2571" max="2574" width="12.85546875" customWidth="1"/>
-    <col min="2575" max="2578" width="12.7109375" customWidth="1"/>
-    <col min="2817" max="2817" width="21.140625" customWidth="1"/>
-    <col min="2818" max="2818" width="12.42578125" customWidth="1"/>
-    <col min="2819" max="2823" width="12.7109375" customWidth="1"/>
-    <col min="2824" max="2824" width="12.85546875" customWidth="1"/>
-    <col min="2825" max="2826" width="12.7109375" customWidth="1"/>
-    <col min="2827" max="2830" width="12.85546875" customWidth="1"/>
-    <col min="2831" max="2834" width="12.7109375" customWidth="1"/>
-    <col min="3073" max="3073" width="21.140625" customWidth="1"/>
-    <col min="3074" max="3074" width="12.42578125" customWidth="1"/>
-    <col min="3075" max="3079" width="12.7109375" customWidth="1"/>
-    <col min="3080" max="3080" width="12.85546875" customWidth="1"/>
-    <col min="3081" max="3082" width="12.7109375" customWidth="1"/>
-    <col min="3083" max="3086" width="12.85546875" customWidth="1"/>
-    <col min="3087" max="3090" width="12.7109375" customWidth="1"/>
-    <col min="3329" max="3329" width="21.140625" customWidth="1"/>
-    <col min="3330" max="3330" width="12.42578125" customWidth="1"/>
-    <col min="3331" max="3335" width="12.7109375" customWidth="1"/>
-    <col min="3336" max="3336" width="12.85546875" customWidth="1"/>
-    <col min="3337" max="3338" width="12.7109375" customWidth="1"/>
-    <col min="3339" max="3342" width="12.85546875" customWidth="1"/>
-    <col min="3343" max="3346" width="12.7109375" customWidth="1"/>
-    <col min="3585" max="3585" width="21.140625" customWidth="1"/>
-    <col min="3586" max="3586" width="12.42578125" customWidth="1"/>
-    <col min="3587" max="3591" width="12.7109375" customWidth="1"/>
-    <col min="3592" max="3592" width="12.85546875" customWidth="1"/>
-    <col min="3593" max="3594" width="12.7109375" customWidth="1"/>
-    <col min="3595" max="3598" width="12.85546875" customWidth="1"/>
-    <col min="3599" max="3602" width="12.7109375" customWidth="1"/>
-    <col min="3841" max="3841" width="21.140625" customWidth="1"/>
-    <col min="3842" max="3842" width="12.42578125" customWidth="1"/>
-    <col min="3843" max="3847" width="12.7109375" customWidth="1"/>
-    <col min="3848" max="3848" width="12.85546875" customWidth="1"/>
-    <col min="3849" max="3850" width="12.7109375" customWidth="1"/>
-    <col min="3851" max="3854" width="12.85546875" customWidth="1"/>
-    <col min="3855" max="3858" width="12.7109375" customWidth="1"/>
-    <col min="4097" max="4097" width="21.140625" customWidth="1"/>
-    <col min="4098" max="4098" width="12.42578125" customWidth="1"/>
-    <col min="4099" max="4103" width="12.7109375" customWidth="1"/>
-    <col min="4104" max="4104" width="12.85546875" customWidth="1"/>
-    <col min="4105" max="4106" width="12.7109375" customWidth="1"/>
-    <col min="4107" max="4110" width="12.85546875" customWidth="1"/>
-    <col min="4111" max="4114" width="12.7109375" customWidth="1"/>
-    <col min="4353" max="4353" width="21.140625" customWidth="1"/>
-    <col min="4354" max="4354" width="12.42578125" customWidth="1"/>
-    <col min="4355" max="4359" width="12.7109375" customWidth="1"/>
-    <col min="4360" max="4360" width="12.85546875" customWidth="1"/>
-    <col min="4361" max="4362" width="12.7109375" customWidth="1"/>
-    <col min="4363" max="4366" width="12.85546875" customWidth="1"/>
-    <col min="4367" max="4370" width="12.7109375" customWidth="1"/>
-    <col min="4609" max="4609" width="21.140625" customWidth="1"/>
-    <col min="4610" max="4610" width="12.42578125" customWidth="1"/>
-    <col min="4611" max="4615" width="12.7109375" customWidth="1"/>
-    <col min="4616" max="4616" width="12.85546875" customWidth="1"/>
-    <col min="4617" max="4618" width="12.7109375" customWidth="1"/>
-    <col min="4619" max="4622" width="12.85546875" customWidth="1"/>
-    <col min="4623" max="4626" width="12.7109375" customWidth="1"/>
-    <col min="4865" max="4865" width="21.140625" customWidth="1"/>
-    <col min="4866" max="4866" width="12.42578125" customWidth="1"/>
-    <col min="4867" max="4871" width="12.7109375" customWidth="1"/>
-    <col min="4872" max="4872" width="12.85546875" customWidth="1"/>
-    <col min="4873" max="4874" width="12.7109375" customWidth="1"/>
-    <col min="4875" max="4878" width="12.85546875" customWidth="1"/>
-    <col min="4879" max="4882" width="12.7109375" customWidth="1"/>
-    <col min="5121" max="5121" width="21.140625" customWidth="1"/>
-    <col min="5122" max="5122" width="12.42578125" customWidth="1"/>
-    <col min="5123" max="5127" width="12.7109375" customWidth="1"/>
-    <col min="5128" max="5128" width="12.85546875" customWidth="1"/>
-    <col min="5129" max="5130" width="12.7109375" customWidth="1"/>
-    <col min="5131" max="5134" width="12.85546875" customWidth="1"/>
-    <col min="5135" max="5138" width="12.7109375" customWidth="1"/>
-    <col min="5377" max="5377" width="21.140625" customWidth="1"/>
-    <col min="5378" max="5378" width="12.42578125" customWidth="1"/>
-    <col min="5379" max="5383" width="12.7109375" customWidth="1"/>
-    <col min="5384" max="5384" width="12.85546875" customWidth="1"/>
-    <col min="5385" max="5386" width="12.7109375" customWidth="1"/>
-    <col min="5387" max="5390" width="12.85546875" customWidth="1"/>
-    <col min="5391" max="5394" width="12.7109375" customWidth="1"/>
-    <col min="5633" max="5633" width="21.140625" customWidth="1"/>
-    <col min="5634" max="5634" width="12.42578125" customWidth="1"/>
-    <col min="5635" max="5639" width="12.7109375" customWidth="1"/>
-    <col min="5640" max="5640" width="12.85546875" customWidth="1"/>
-    <col min="5641" max="5642" width="12.7109375" customWidth="1"/>
-    <col min="5643" max="5646" width="12.85546875" customWidth="1"/>
-    <col min="5647" max="5650" width="12.7109375" customWidth="1"/>
-    <col min="5889" max="5889" width="21.140625" customWidth="1"/>
-    <col min="5890" max="5890" width="12.42578125" customWidth="1"/>
-    <col min="5891" max="5895" width="12.7109375" customWidth="1"/>
-    <col min="5896" max="5896" width="12.85546875" customWidth="1"/>
-    <col min="5897" max="5898" width="12.7109375" customWidth="1"/>
-    <col min="5899" max="5902" width="12.85546875" customWidth="1"/>
-    <col min="5903" max="5906" width="12.7109375" customWidth="1"/>
-    <col min="6145" max="6145" width="21.140625" customWidth="1"/>
-    <col min="6146" max="6146" width="12.42578125" customWidth="1"/>
-    <col min="6147" max="6151" width="12.7109375" customWidth="1"/>
-    <col min="6152" max="6152" width="12.85546875" customWidth="1"/>
-    <col min="6153" max="6154" width="12.7109375" customWidth="1"/>
-    <col min="6155" max="6158" width="12.85546875" customWidth="1"/>
-    <col min="6159" max="6162" width="12.7109375" customWidth="1"/>
-    <col min="6401" max="6401" width="21.140625" customWidth="1"/>
-    <col min="6402" max="6402" width="12.42578125" customWidth="1"/>
-    <col min="6403" max="6407" width="12.7109375" customWidth="1"/>
-    <col min="6408" max="6408" width="12.85546875" customWidth="1"/>
-    <col min="6409" max="6410" width="12.7109375" customWidth="1"/>
-    <col min="6411" max="6414" width="12.85546875" customWidth="1"/>
-    <col min="6415" max="6418" width="12.7109375" customWidth="1"/>
-    <col min="6657" max="6657" width="21.140625" customWidth="1"/>
-    <col min="6658" max="6658" width="12.42578125" customWidth="1"/>
-    <col min="6659" max="6663" width="12.7109375" customWidth="1"/>
-    <col min="6664" max="6664" width="12.85546875" customWidth="1"/>
-    <col min="6665" max="6666" width="12.7109375" customWidth="1"/>
-    <col min="6667" max="6670" width="12.85546875" customWidth="1"/>
-    <col min="6671" max="6674" width="12.7109375" customWidth="1"/>
-    <col min="6913" max="6913" width="21.140625" customWidth="1"/>
-    <col min="6914" max="6914" width="12.42578125" customWidth="1"/>
-    <col min="6915" max="6919" width="12.7109375" customWidth="1"/>
-    <col min="6920" max="6920" width="12.85546875" customWidth="1"/>
-    <col min="6921" max="6922" width="12.7109375" customWidth="1"/>
-    <col min="6923" max="6926" width="12.85546875" customWidth="1"/>
-    <col min="6927" max="6930" width="12.7109375" customWidth="1"/>
-    <col min="7169" max="7169" width="21.140625" customWidth="1"/>
-    <col min="7170" max="7170" width="12.42578125" customWidth="1"/>
-    <col min="7171" max="7175" width="12.7109375" customWidth="1"/>
-    <col min="7176" max="7176" width="12.85546875" customWidth="1"/>
-    <col min="7177" max="7178" width="12.7109375" customWidth="1"/>
-    <col min="7179" max="7182" width="12.85546875" customWidth="1"/>
-    <col min="7183" max="7186" width="12.7109375" customWidth="1"/>
-    <col min="7425" max="7425" width="21.140625" customWidth="1"/>
-    <col min="7426" max="7426" width="12.42578125" customWidth="1"/>
-    <col min="7427" max="7431" width="12.7109375" customWidth="1"/>
-    <col min="7432" max="7432" width="12.85546875" customWidth="1"/>
-    <col min="7433" max="7434" width="12.7109375" customWidth="1"/>
-    <col min="7435" max="7438" width="12.85546875" customWidth="1"/>
-    <col min="7439" max="7442" width="12.7109375" customWidth="1"/>
-    <col min="7681" max="7681" width="21.140625" customWidth="1"/>
-    <col min="7682" max="7682" width="12.42578125" customWidth="1"/>
-    <col min="7683" max="7687" width="12.7109375" customWidth="1"/>
-    <col min="7688" max="7688" width="12.85546875" customWidth="1"/>
-    <col min="7689" max="7690" width="12.7109375" customWidth="1"/>
-    <col min="7691" max="7694" width="12.85546875" customWidth="1"/>
-    <col min="7695" max="7698" width="12.7109375" customWidth="1"/>
-    <col min="7937" max="7937" width="21.140625" customWidth="1"/>
-    <col min="7938" max="7938" width="12.42578125" customWidth="1"/>
-    <col min="7939" max="7943" width="12.7109375" customWidth="1"/>
-    <col min="7944" max="7944" width="12.85546875" customWidth="1"/>
-    <col min="7945" max="7946" width="12.7109375" customWidth="1"/>
-    <col min="7947" max="7950" width="12.85546875" customWidth="1"/>
-    <col min="7951" max="7954" width="12.7109375" customWidth="1"/>
-    <col min="8193" max="8193" width="21.140625" customWidth="1"/>
-    <col min="8194" max="8194" width="12.42578125" customWidth="1"/>
-    <col min="8195" max="8199" width="12.7109375" customWidth="1"/>
-    <col min="8200" max="8200" width="12.85546875" customWidth="1"/>
-    <col min="8201" max="8202" width="12.7109375" customWidth="1"/>
-    <col min="8203" max="8206" width="12.85546875" customWidth="1"/>
-    <col min="8207" max="8210" width="12.7109375" customWidth="1"/>
-    <col min="8449" max="8449" width="21.140625" customWidth="1"/>
-    <col min="8450" max="8450" width="12.42578125" customWidth="1"/>
-    <col min="8451" max="8455" width="12.7109375" customWidth="1"/>
-    <col min="8456" max="8456" width="12.85546875" customWidth="1"/>
-    <col min="8457" max="8458" width="12.7109375" customWidth="1"/>
-    <col min="8459" max="8462" width="12.85546875" customWidth="1"/>
-    <col min="8463" max="8466" width="12.7109375" customWidth="1"/>
-    <col min="8705" max="8705" width="21.140625" customWidth="1"/>
-    <col min="8706" max="8706" width="12.42578125" customWidth="1"/>
-    <col min="8707" max="8711" width="12.7109375" customWidth="1"/>
-    <col min="8712" max="8712" width="12.85546875" customWidth="1"/>
-    <col min="8713" max="8714" width="12.7109375" customWidth="1"/>
-    <col min="8715" max="8718" width="12.85546875" customWidth="1"/>
-    <col min="8719" max="8722" width="12.7109375" customWidth="1"/>
-    <col min="8961" max="8961" width="21.140625" customWidth="1"/>
-    <col min="8962" max="8962" width="12.42578125" customWidth="1"/>
-    <col min="8963" max="8967" width="12.7109375" customWidth="1"/>
-    <col min="8968" max="8968" width="12.85546875" customWidth="1"/>
-    <col min="8969" max="8970" width="12.7109375" customWidth="1"/>
-    <col min="8971" max="8974" width="12.85546875" customWidth="1"/>
-    <col min="8975" max="8978" width="12.7109375" customWidth="1"/>
-    <col min="9217" max="9217" width="21.140625" customWidth="1"/>
-    <col min="9218" max="9218" width="12.42578125" customWidth="1"/>
-    <col min="9219" max="9223" width="12.7109375" customWidth="1"/>
-    <col min="9224" max="9224" width="12.85546875" customWidth="1"/>
-    <col min="9225" max="9226" width="12.7109375" customWidth="1"/>
-    <col min="9227" max="9230" width="12.85546875" customWidth="1"/>
-    <col min="9231" max="9234" width="12.7109375" customWidth="1"/>
-    <col min="9473" max="9473" width="21.140625" customWidth="1"/>
-    <col min="9474" max="9474" width="12.42578125" customWidth="1"/>
-    <col min="9475" max="9479" width="12.7109375" customWidth="1"/>
-    <col min="9480" max="9480" width="12.85546875" customWidth="1"/>
-    <col min="9481" max="9482" width="12.7109375" customWidth="1"/>
-    <col min="9483" max="9486" width="12.85546875" customWidth="1"/>
-    <col min="9487" max="9490" width="12.7109375" customWidth="1"/>
-    <col min="9729" max="9729" width="21.140625" customWidth="1"/>
-    <col min="9730" max="9730" width="12.42578125" customWidth="1"/>
-    <col min="9731" max="9735" width="12.7109375" customWidth="1"/>
-    <col min="9736" max="9736" width="12.85546875" customWidth="1"/>
-    <col min="9737" max="9738" width="12.7109375" customWidth="1"/>
-    <col min="9739" max="9742" width="12.85546875" customWidth="1"/>
-    <col min="9743" max="9746" width="12.7109375" customWidth="1"/>
-    <col min="9985" max="9985" width="21.140625" customWidth="1"/>
-    <col min="9986" max="9986" width="12.42578125" customWidth="1"/>
-    <col min="9987" max="9991" width="12.7109375" customWidth="1"/>
-    <col min="9992" max="9992" width="12.85546875" customWidth="1"/>
-    <col min="9993" max="9994" width="12.7109375" customWidth="1"/>
-    <col min="9995" max="9998" width="12.85546875" customWidth="1"/>
-    <col min="9999" max="10002" width="12.7109375" customWidth="1"/>
-    <col min="10241" max="10241" width="21.140625" customWidth="1"/>
-    <col min="10242" max="10242" width="12.42578125" customWidth="1"/>
-    <col min="10243" max="10247" width="12.7109375" customWidth="1"/>
-    <col min="10248" max="10248" width="12.85546875" customWidth="1"/>
-    <col min="10249" max="10250" width="12.7109375" customWidth="1"/>
-    <col min="10251" max="10254" width="12.85546875" customWidth="1"/>
-    <col min="10255" max="10258" width="12.7109375" customWidth="1"/>
-    <col min="10497" max="10497" width="21.140625" customWidth="1"/>
-    <col min="10498" max="10498" width="12.42578125" customWidth="1"/>
-    <col min="10499" max="10503" width="12.7109375" customWidth="1"/>
-    <col min="10504" max="10504" width="12.85546875" customWidth="1"/>
-    <col min="10505" max="10506" width="12.7109375" customWidth="1"/>
-    <col min="10507" max="10510" width="12.85546875" customWidth="1"/>
-    <col min="10511" max="10514" width="12.7109375" customWidth="1"/>
-    <col min="10753" max="10753" width="21.140625" customWidth="1"/>
-    <col min="10754" max="10754" width="12.42578125" customWidth="1"/>
-    <col min="10755" max="10759" width="12.7109375" customWidth="1"/>
-    <col min="10760" max="10760" width="12.85546875" customWidth="1"/>
-    <col min="10761" max="10762" width="12.7109375" customWidth="1"/>
-    <col min="10763" max="10766" width="12.85546875" customWidth="1"/>
-    <col min="10767" max="10770" width="12.7109375" customWidth="1"/>
-    <col min="11009" max="11009" width="21.140625" customWidth="1"/>
-    <col min="11010" max="11010" width="12.42578125" customWidth="1"/>
-    <col min="11011" max="11015" width="12.7109375" customWidth="1"/>
-    <col min="11016" max="11016" width="12.85546875" customWidth="1"/>
-    <col min="11017" max="11018" width="12.7109375" customWidth="1"/>
-    <col min="11019" max="11022" width="12.85546875" customWidth="1"/>
-    <col min="11023" max="11026" width="12.7109375" customWidth="1"/>
-    <col min="11265" max="11265" width="21.140625" customWidth="1"/>
-    <col min="11266" max="11266" width="12.42578125" customWidth="1"/>
-    <col min="11267" max="11271" width="12.7109375" customWidth="1"/>
-    <col min="11272" max="11272" width="12.85546875" customWidth="1"/>
-    <col min="11273" max="11274" width="12.7109375" customWidth="1"/>
-    <col min="11275" max="11278" width="12.85546875" customWidth="1"/>
-    <col min="11279" max="11282" width="12.7109375" customWidth="1"/>
-    <col min="11521" max="11521" width="21.140625" customWidth="1"/>
-    <col min="11522" max="11522" width="12.42578125" customWidth="1"/>
-    <col min="11523" max="11527" width="12.7109375" customWidth="1"/>
-    <col min="11528" max="11528" width="12.85546875" customWidth="1"/>
-    <col min="11529" max="11530" width="12.7109375" customWidth="1"/>
-    <col min="11531" max="11534" width="12.85546875" customWidth="1"/>
-    <col min="11535" max="11538" width="12.7109375" customWidth="1"/>
-    <col min="11777" max="11777" width="21.140625" customWidth="1"/>
-    <col min="11778" max="11778" width="12.42578125" customWidth="1"/>
-    <col min="11779" max="11783" width="12.7109375" customWidth="1"/>
-    <col min="11784" max="11784" width="12.85546875" customWidth="1"/>
-    <col min="11785" max="11786" width="12.7109375" customWidth="1"/>
-    <col min="11787" max="11790" width="12.85546875" customWidth="1"/>
-    <col min="11791" max="11794" width="12.7109375" customWidth="1"/>
-    <col min="12033" max="12033" width="21.140625" customWidth="1"/>
-    <col min="12034" max="12034" width="12.42578125" customWidth="1"/>
-    <col min="12035" max="12039" width="12.7109375" customWidth="1"/>
-    <col min="12040" max="12040" width="12.85546875" customWidth="1"/>
-    <col min="12041" max="12042" width="12.7109375" customWidth="1"/>
-    <col min="12043" max="12046" width="12.85546875" customWidth="1"/>
-    <col min="12047" max="12050" width="12.7109375" customWidth="1"/>
-    <col min="12289" max="12289" width="21.140625" customWidth="1"/>
-    <col min="12290" max="12290" width="12.42578125" customWidth="1"/>
-    <col min="12291" max="12295" width="12.7109375" customWidth="1"/>
-    <col min="12296" max="12296" width="12.85546875" customWidth="1"/>
-    <col min="12297" max="12298" width="12.7109375" customWidth="1"/>
-    <col min="12299" max="12302" width="12.85546875" customWidth="1"/>
-    <col min="12303" max="12306" width="12.7109375" customWidth="1"/>
-    <col min="12545" max="12545" width="21.140625" customWidth="1"/>
-    <col min="12546" max="12546" width="12.42578125" customWidth="1"/>
-    <col min="12547" max="12551" width="12.7109375" customWidth="1"/>
-    <col min="12552" max="12552" width="12.85546875" customWidth="1"/>
-    <col min="12553" max="12554" width="12.7109375" customWidth="1"/>
-    <col min="12555" max="12558" width="12.85546875" customWidth="1"/>
-    <col min="12559" max="12562" width="12.7109375" customWidth="1"/>
-    <col min="12801" max="12801" width="21.140625" customWidth="1"/>
-    <col min="12802" max="12802" width="12.42578125" customWidth="1"/>
-    <col min="12803" max="12807" width="12.7109375" customWidth="1"/>
-    <col min="12808" max="12808" width="12.85546875" customWidth="1"/>
-    <col min="12809" max="12810" width="12.7109375" customWidth="1"/>
-    <col min="12811" max="12814" width="12.85546875" customWidth="1"/>
-    <col min="12815" max="12818" width="12.7109375" customWidth="1"/>
-    <col min="13057" max="13057" width="21.140625" customWidth="1"/>
-    <col min="13058" max="13058" width="12.42578125" customWidth="1"/>
-    <col min="13059" max="13063" width="12.7109375" customWidth="1"/>
-    <col min="13064" max="13064" width="12.85546875" customWidth="1"/>
-    <col min="13065" max="13066" width="12.7109375" customWidth="1"/>
-    <col min="13067" max="13070" width="12.85546875" customWidth="1"/>
-    <col min="13071" max="13074" width="12.7109375" customWidth="1"/>
-    <col min="13313" max="13313" width="21.140625" customWidth="1"/>
-    <col min="13314" max="13314" width="12.42578125" customWidth="1"/>
-    <col min="13315" max="13319" width="12.7109375" customWidth="1"/>
-    <col min="13320" max="13320" width="12.85546875" customWidth="1"/>
-    <col min="13321" max="13322" width="12.7109375" customWidth="1"/>
-    <col min="13323" max="13326" width="12.85546875" customWidth="1"/>
-    <col min="13327" max="13330" width="12.7109375" customWidth="1"/>
-    <col min="13569" max="13569" width="21.140625" customWidth="1"/>
-    <col min="13570" max="13570" width="12.42578125" customWidth="1"/>
-    <col min="13571" max="13575" width="12.7109375" customWidth="1"/>
-    <col min="13576" max="13576" width="12.85546875" customWidth="1"/>
-    <col min="13577" max="13578" width="12.7109375" customWidth="1"/>
-    <col min="13579" max="13582" width="12.85546875" customWidth="1"/>
-    <col min="13583" max="13586" width="12.7109375" customWidth="1"/>
-    <col min="13825" max="13825" width="21.140625" customWidth="1"/>
-    <col min="13826" max="13826" width="12.42578125" customWidth="1"/>
-    <col min="13827" max="13831" width="12.7109375" customWidth="1"/>
-    <col min="13832" max="13832" width="12.85546875" customWidth="1"/>
-    <col min="13833" max="13834" width="12.7109375" customWidth="1"/>
-    <col min="13835" max="13838" width="12.85546875" customWidth="1"/>
-    <col min="13839" max="13842" width="12.7109375" customWidth="1"/>
-    <col min="14081" max="14081" width="21.140625" customWidth="1"/>
-    <col min="14082" max="14082" width="12.42578125" customWidth="1"/>
-    <col min="14083" max="14087" width="12.7109375" customWidth="1"/>
-    <col min="14088" max="14088" width="12.85546875" customWidth="1"/>
-    <col min="14089" max="14090" width="12.7109375" customWidth="1"/>
-    <col min="14091" max="14094" width="12.85546875" customWidth="1"/>
-    <col min="14095" max="14098" width="12.7109375" customWidth="1"/>
-    <col min="14337" max="14337" width="21.140625" customWidth="1"/>
-    <col min="14338" max="14338" width="12.42578125" customWidth="1"/>
-    <col min="14339" max="14343" width="12.7109375" customWidth="1"/>
-    <col min="14344" max="14344" width="12.85546875" customWidth="1"/>
-    <col min="14345" max="14346" width="12.7109375" customWidth="1"/>
-    <col min="14347" max="14350" width="12.85546875" customWidth="1"/>
-    <col min="14351" max="14354" width="12.7109375" customWidth="1"/>
-    <col min="14593" max="14593" width="21.140625" customWidth="1"/>
-    <col min="14594" max="14594" width="12.42578125" customWidth="1"/>
-    <col min="14595" max="14599" width="12.7109375" customWidth="1"/>
-    <col min="14600" max="14600" width="12.85546875" customWidth="1"/>
-    <col min="14601" max="14602" width="12.7109375" customWidth="1"/>
-    <col min="14603" max="14606" width="12.85546875" customWidth="1"/>
-    <col min="14607" max="14610" width="12.7109375" customWidth="1"/>
-    <col min="14849" max="14849" width="21.140625" customWidth="1"/>
-    <col min="14850" max="14850" width="12.42578125" customWidth="1"/>
-    <col min="14851" max="14855" width="12.7109375" customWidth="1"/>
-    <col min="14856" max="14856" width="12.85546875" customWidth="1"/>
-    <col min="14857" max="14858" width="12.7109375" customWidth="1"/>
-    <col min="14859" max="14862" width="12.85546875" customWidth="1"/>
-    <col min="14863" max="14866" width="12.7109375" customWidth="1"/>
-    <col min="15105" max="15105" width="21.140625" customWidth="1"/>
-    <col min="15106" max="15106" width="12.42578125" customWidth="1"/>
-    <col min="15107" max="15111" width="12.7109375" customWidth="1"/>
-    <col min="15112" max="15112" width="12.85546875" customWidth="1"/>
-    <col min="15113" max="15114" width="12.7109375" customWidth="1"/>
-    <col min="15115" max="15118" width="12.85546875" customWidth="1"/>
-    <col min="15119" max="15122" width="12.7109375" customWidth="1"/>
-    <col min="15361" max="15361" width="21.140625" customWidth="1"/>
-    <col min="15362" max="15362" width="12.42578125" customWidth="1"/>
-    <col min="15363" max="15367" width="12.7109375" customWidth="1"/>
-    <col min="15368" max="15368" width="12.85546875" customWidth="1"/>
-    <col min="15369" max="15370" width="12.7109375" customWidth="1"/>
-    <col min="15371" max="15374" width="12.85546875" customWidth="1"/>
-    <col min="15375" max="15378" width="12.7109375" customWidth="1"/>
-    <col min="15617" max="15617" width="21.140625" customWidth="1"/>
-    <col min="15618" max="15618" width="12.42578125" customWidth="1"/>
-    <col min="15619" max="15623" width="12.7109375" customWidth="1"/>
-    <col min="15624" max="15624" width="12.85546875" customWidth="1"/>
-    <col min="15625" max="15626" width="12.7109375" customWidth="1"/>
-    <col min="15627" max="15630" width="12.85546875" customWidth="1"/>
-    <col min="15631" max="15634" width="12.7109375" customWidth="1"/>
-    <col min="15873" max="15873" width="21.140625" customWidth="1"/>
-    <col min="15874" max="15874" width="12.42578125" customWidth="1"/>
-    <col min="15875" max="15879" width="12.7109375" customWidth="1"/>
-    <col min="15880" max="15880" width="12.85546875" customWidth="1"/>
-    <col min="15881" max="15882" width="12.7109375" customWidth="1"/>
-    <col min="15883" max="15886" width="12.85546875" customWidth="1"/>
-    <col min="15887" max="15890" width="12.7109375" customWidth="1"/>
-    <col min="16129" max="16129" width="21.140625" customWidth="1"/>
-    <col min="16130" max="16130" width="12.42578125" customWidth="1"/>
-    <col min="16131" max="16135" width="12.7109375" customWidth="1"/>
-    <col min="16136" max="16136" width="12.85546875" customWidth="1"/>
-    <col min="16137" max="16138" width="12.7109375" customWidth="1"/>
-    <col min="16139" max="16142" width="12.85546875" customWidth="1"/>
-    <col min="16143" max="16146" width="12.7109375" customWidth="1"/>
+    <col min="1" max="1" width="21.1796875" customWidth="1"/>
+    <col min="2" max="2" width="12.453125" customWidth="1"/>
+    <col min="3" max="7" width="12.7265625" customWidth="1"/>
+    <col min="8" max="8" width="12.81640625" customWidth="1"/>
+    <col min="9" max="10" width="12.7265625" customWidth="1"/>
+    <col min="11" max="14" width="12.81640625" customWidth="1"/>
+    <col min="15" max="18" width="12.7265625" customWidth="1"/>
+    <col min="257" max="257" width="21.1796875" customWidth="1"/>
+    <col min="258" max="258" width="12.453125" customWidth="1"/>
+    <col min="259" max="263" width="12.7265625" customWidth="1"/>
+    <col min="264" max="264" width="12.81640625" customWidth="1"/>
+    <col min="265" max="266" width="12.7265625" customWidth="1"/>
+    <col min="267" max="270" width="12.81640625" customWidth="1"/>
+    <col min="271" max="274" width="12.7265625" customWidth="1"/>
+    <col min="513" max="513" width="21.1796875" customWidth="1"/>
+    <col min="514" max="514" width="12.453125" customWidth="1"/>
+    <col min="515" max="519" width="12.7265625" customWidth="1"/>
+    <col min="520" max="520" width="12.81640625" customWidth="1"/>
+    <col min="521" max="522" width="12.7265625" customWidth="1"/>
+    <col min="523" max="526" width="12.81640625" customWidth="1"/>
+    <col min="527" max="530" width="12.7265625" customWidth="1"/>
+    <col min="769" max="769" width="21.1796875" customWidth="1"/>
+    <col min="770" max="770" width="12.453125" customWidth="1"/>
+    <col min="771" max="775" width="12.7265625" customWidth="1"/>
+    <col min="776" max="776" width="12.81640625" customWidth="1"/>
+    <col min="777" max="778" width="12.7265625" customWidth="1"/>
+    <col min="779" max="782" width="12.81640625" customWidth="1"/>
+    <col min="783" max="786" width="12.7265625" customWidth="1"/>
+    <col min="1025" max="1025" width="21.1796875" customWidth="1"/>
+    <col min="1026" max="1026" width="12.453125" customWidth="1"/>
+    <col min="1027" max="1031" width="12.7265625" customWidth="1"/>
+    <col min="1032" max="1032" width="12.81640625" customWidth="1"/>
+    <col min="1033" max="1034" width="12.7265625" customWidth="1"/>
+    <col min="1035" max="1038" width="12.81640625" customWidth="1"/>
+    <col min="1039" max="1042" width="12.7265625" customWidth="1"/>
+    <col min="1281" max="1281" width="21.1796875" customWidth="1"/>
+    <col min="1282" max="1282" width="12.453125" customWidth="1"/>
+    <col min="1283" max="1287" width="12.7265625" customWidth="1"/>
+    <col min="1288" max="1288" width="12.81640625" customWidth="1"/>
+    <col min="1289" max="1290" width="12.7265625" customWidth="1"/>
+    <col min="1291" max="1294" width="12.81640625" customWidth="1"/>
+    <col min="1295" max="1298" width="12.7265625" customWidth="1"/>
+    <col min="1537" max="1537" width="21.1796875" customWidth="1"/>
+    <col min="1538" max="1538" width="12.453125" customWidth="1"/>
+    <col min="1539" max="1543" width="12.7265625" customWidth="1"/>
+    <col min="1544" max="1544" width="12.81640625" customWidth="1"/>
+    <col min="1545" max="1546" width="12.7265625" customWidth="1"/>
+    <col min="1547" max="1550" width="12.81640625" customWidth="1"/>
+    <col min="1551" max="1554" width="12.7265625" customWidth="1"/>
+    <col min="1793" max="1793" width="21.1796875" customWidth="1"/>
+    <col min="1794" max="1794" width="12.453125" customWidth="1"/>
+    <col min="1795" max="1799" width="12.7265625" customWidth="1"/>
+    <col min="1800" max="1800" width="12.81640625" customWidth="1"/>
+    <col min="1801" max="1802" width="12.7265625" customWidth="1"/>
+    <col min="1803" max="1806" width="12.81640625" customWidth="1"/>
+    <col min="1807" max="1810" width="12.7265625" customWidth="1"/>
+    <col min="2049" max="2049" width="21.1796875" customWidth="1"/>
+    <col min="2050" max="2050" width="12.453125" customWidth="1"/>
+    <col min="2051" max="2055" width="12.7265625" customWidth="1"/>
+    <col min="2056" max="2056" width="12.81640625" customWidth="1"/>
+    <col min="2057" max="2058" width="12.7265625" customWidth="1"/>
+    <col min="2059" max="2062" width="12.81640625" customWidth="1"/>
+    <col min="2063" max="2066" width="12.7265625" customWidth="1"/>
+    <col min="2305" max="2305" width="21.1796875" customWidth="1"/>
+    <col min="2306" max="2306" width="12.453125" customWidth="1"/>
+    <col min="2307" max="2311" width="12.7265625" customWidth="1"/>
+    <col min="2312" max="2312" width="12.81640625" customWidth="1"/>
+    <col min="2313" max="2314" width="12.7265625" customWidth="1"/>
+    <col min="2315" max="2318" width="12.81640625" customWidth="1"/>
+    <col min="2319" max="2322" width="12.7265625" customWidth="1"/>
+    <col min="2561" max="2561" width="21.1796875" customWidth="1"/>
+    <col min="2562" max="2562" width="12.453125" customWidth="1"/>
+    <col min="2563" max="2567" width="12.7265625" customWidth="1"/>
+    <col min="2568" max="2568" width="12.81640625" customWidth="1"/>
+    <col min="2569" max="2570" width="12.7265625" customWidth="1"/>
+    <col min="2571" max="2574" width="12.81640625" customWidth="1"/>
+    <col min="2575" max="2578" width="12.7265625" customWidth="1"/>
+    <col min="2817" max="2817" width="21.1796875" customWidth="1"/>
+    <col min="2818" max="2818" width="12.453125" customWidth="1"/>
+    <col min="2819" max="2823" width="12.7265625" customWidth="1"/>
+    <col min="2824" max="2824" width="12.81640625" customWidth="1"/>
+    <col min="2825" max="2826" width="12.7265625" customWidth="1"/>
+    <col min="2827" max="2830" width="12.81640625" customWidth="1"/>
+    <col min="2831" max="2834" width="12.7265625" customWidth="1"/>
+    <col min="3073" max="3073" width="21.1796875" customWidth="1"/>
+    <col min="3074" max="3074" width="12.453125" customWidth="1"/>
+    <col min="3075" max="3079" width="12.7265625" customWidth="1"/>
+    <col min="3080" max="3080" width="12.81640625" customWidth="1"/>
+    <col min="3081" max="3082" width="12.7265625" customWidth="1"/>
+    <col min="3083" max="3086" width="12.81640625" customWidth="1"/>
+    <col min="3087" max="3090" width="12.7265625" customWidth="1"/>
+    <col min="3329" max="3329" width="21.1796875" customWidth="1"/>
+    <col min="3330" max="3330" width="12.453125" customWidth="1"/>
+    <col min="3331" max="3335" width="12.7265625" customWidth="1"/>
+    <col min="3336" max="3336" width="12.81640625" customWidth="1"/>
+    <col min="3337" max="3338" width="12.7265625" customWidth="1"/>
+    <col min="3339" max="3342" width="12.81640625" customWidth="1"/>
+    <col min="3343" max="3346" width="12.7265625" customWidth="1"/>
+    <col min="3585" max="3585" width="21.1796875" customWidth="1"/>
+    <col min="3586" max="3586" width="12.453125" customWidth="1"/>
+    <col min="3587" max="3591" width="12.7265625" customWidth="1"/>
+    <col min="3592" max="3592" width="12.81640625" customWidth="1"/>
+    <col min="3593" max="3594" width="12.7265625" customWidth="1"/>
+    <col min="3595" max="3598" width="12.81640625" customWidth="1"/>
+    <col min="3599" max="3602" width="12.7265625" customWidth="1"/>
+    <col min="3841" max="3841" width="21.1796875" customWidth="1"/>
+    <col min="3842" max="3842" width="12.453125" customWidth="1"/>
+    <col min="3843" max="3847" width="12.7265625" customWidth="1"/>
+    <col min="3848" max="3848" width="12.81640625" customWidth="1"/>
+    <col min="3849" max="3850" width="12.7265625" customWidth="1"/>
+    <col min="3851" max="3854" width="12.81640625" customWidth="1"/>
+    <col min="3855" max="3858" width="12.7265625" customWidth="1"/>
+    <col min="4097" max="4097" width="21.1796875" customWidth="1"/>
+    <col min="4098" max="4098" width="12.453125" customWidth="1"/>
+    <col min="4099" max="4103" width="12.7265625" customWidth="1"/>
+    <col min="4104" max="4104" width="12.81640625" customWidth="1"/>
+    <col min="4105" max="4106" width="12.7265625" customWidth="1"/>
+    <col min="4107" max="4110" width="12.81640625" customWidth="1"/>
+    <col min="4111" max="4114" width="12.7265625" customWidth="1"/>
+    <col min="4353" max="4353" width="21.1796875" customWidth="1"/>
+    <col min="4354" max="4354" width="12.453125" customWidth="1"/>
+    <col min="4355" max="4359" width="12.7265625" customWidth="1"/>
+    <col min="4360" max="4360" width="12.81640625" customWidth="1"/>
+    <col min="4361" max="4362" width="12.7265625" customWidth="1"/>
+    <col min="4363" max="4366" width="12.81640625" customWidth="1"/>
+    <col min="4367" max="4370" width="12.7265625" customWidth="1"/>
+    <col min="4609" max="4609" width="21.1796875" customWidth="1"/>
+    <col min="4610" max="4610" width="12.453125" customWidth="1"/>
+    <col min="4611" max="4615" width="12.7265625" customWidth="1"/>
+    <col min="4616" max="4616" width="12.81640625" customWidth="1"/>
+    <col min="4617" max="4618" width="12.7265625" customWidth="1"/>
+    <col min="4619" max="4622" width="12.81640625" customWidth="1"/>
+    <col min="4623" max="4626" width="12.7265625" customWidth="1"/>
+    <col min="4865" max="4865" width="21.1796875" customWidth="1"/>
+    <col min="4866" max="4866" width="12.453125" customWidth="1"/>
+    <col min="4867" max="4871" width="12.7265625" customWidth="1"/>
+    <col min="4872" max="4872" width="12.81640625" customWidth="1"/>
+    <col min="4873" max="4874" width="12.7265625" customWidth="1"/>
+    <col min="4875" max="4878" width="12.81640625" customWidth="1"/>
+    <col min="4879" max="4882" width="12.7265625" customWidth="1"/>
+    <col min="5121" max="5121" width="21.1796875" customWidth="1"/>
+    <col min="5122" max="5122" width="12.453125" customWidth="1"/>
+    <col min="5123" max="5127" width="12.7265625" customWidth="1"/>
+    <col min="5128" max="5128" width="12.81640625" customWidth="1"/>
+    <col min="5129" max="5130" width="12.7265625" customWidth="1"/>
+    <col min="5131" max="5134" width="12.81640625" customWidth="1"/>
+    <col min="5135" max="5138" width="12.7265625" customWidth="1"/>
+    <col min="5377" max="5377" width="21.1796875" customWidth="1"/>
+    <col min="5378" max="5378" width="12.453125" customWidth="1"/>
+    <col min="5379" max="5383" width="12.7265625" customWidth="1"/>
+    <col min="5384" max="5384" width="12.81640625" customWidth="1"/>
+    <col min="5385" max="5386" width="12.7265625" customWidth="1"/>
+    <col min="5387" max="5390" width="12.81640625" customWidth="1"/>
+    <col min="5391" max="5394" width="12.7265625" customWidth="1"/>
+    <col min="5633" max="5633" width="21.1796875" customWidth="1"/>
+    <col min="5634" max="5634" width="12.453125" customWidth="1"/>
+    <col min="5635" max="5639" width="12.7265625" customWidth="1"/>
+    <col min="5640" max="5640" width="12.81640625" customWidth="1"/>
+    <col min="5641" max="5642" width="12.7265625" customWidth="1"/>
+    <col min="5643" max="5646" width="12.81640625" customWidth="1"/>
+    <col min="5647" max="5650" width="12.7265625" customWidth="1"/>
+    <col min="5889" max="5889" width="21.1796875" customWidth="1"/>
+    <col min="5890" max="5890" width="12.453125" customWidth="1"/>
+    <col min="5891" max="5895" width="12.7265625" customWidth="1"/>
+    <col min="5896" max="5896" width="12.81640625" customWidth="1"/>
+    <col min="5897" max="5898" width="12.7265625" customWidth="1"/>
+    <col min="5899" max="5902" width="12.81640625" customWidth="1"/>
+    <col min="5903" max="5906" width="12.7265625" customWidth="1"/>
+    <col min="6145" max="6145" width="21.1796875" customWidth="1"/>
+    <col min="6146" max="6146" width="12.453125" customWidth="1"/>
+    <col min="6147" max="6151" width="12.7265625" customWidth="1"/>
+    <col min="6152" max="6152" width="12.81640625" customWidth="1"/>
+    <col min="6153" max="6154" width="12.7265625" customWidth="1"/>
+    <col min="6155" max="6158" width="12.81640625" customWidth="1"/>
+    <col min="6159" max="6162" width="12.7265625" customWidth="1"/>
+    <col min="6401" max="6401" width="21.1796875" customWidth="1"/>
+    <col min="6402" max="6402" width="12.453125" customWidth="1"/>
+    <col min="6403" max="6407" width="12.7265625" customWidth="1"/>
+    <col min="6408" max="6408" width="12.81640625" customWidth="1"/>
+    <col min="6409" max="6410" width="12.7265625" customWidth="1"/>
+    <col min="6411" max="6414" width="12.81640625" customWidth="1"/>
+    <col min="6415" max="6418" width="12.7265625" customWidth="1"/>
+    <col min="6657" max="6657" width="21.1796875" customWidth="1"/>
+    <col min="6658" max="6658" width="12.453125" customWidth="1"/>
+    <col min="6659" max="6663" width="12.7265625" customWidth="1"/>
+    <col min="6664" max="6664" width="12.81640625" customWidth="1"/>
+    <col min="6665" max="6666" width="12.7265625" customWidth="1"/>
+    <col min="6667" max="6670" width="12.81640625" customWidth="1"/>
+    <col min="6671" max="6674" width="12.7265625" customWidth="1"/>
+    <col min="6913" max="6913" width="21.1796875" customWidth="1"/>
+    <col min="6914" max="6914" width="12.453125" customWidth="1"/>
+    <col min="6915" max="6919" width="12.7265625" customWidth="1"/>
+    <col min="6920" max="6920" width="12.81640625" customWidth="1"/>
+    <col min="6921" max="6922" width="12.7265625" customWidth="1"/>
+    <col min="6923" max="6926" width="12.81640625" customWidth="1"/>
+    <col min="6927" max="6930" width="12.7265625" customWidth="1"/>
+    <col min="7169" max="7169" width="21.1796875" customWidth="1"/>
+    <col min="7170" max="7170" width="12.453125" customWidth="1"/>
+    <col min="7171" max="7175" width="12.7265625" customWidth="1"/>
+    <col min="7176" max="7176" width="12.81640625" customWidth="1"/>
+    <col min="7177" max="7178" width="12.7265625" customWidth="1"/>
+    <col min="7179" max="7182" width="12.81640625" customWidth="1"/>
+    <col min="7183" max="7186" width="12.7265625" customWidth="1"/>
+    <col min="7425" max="7425" width="21.1796875" customWidth="1"/>
+    <col min="7426" max="7426" width="12.453125" customWidth="1"/>
+    <col min="7427" max="7431" width="12.7265625" customWidth="1"/>
+    <col min="7432" max="7432" width="12.81640625" customWidth="1"/>
+    <col min="7433" max="7434" width="12.7265625" customWidth="1"/>
+    <col min="7435" max="7438" width="12.81640625" customWidth="1"/>
+    <col min="7439" max="7442" width="12.7265625" customWidth="1"/>
+    <col min="7681" max="7681" width="21.1796875" customWidth="1"/>
+    <col min="7682" max="7682" width="12.453125" customWidth="1"/>
+    <col min="7683" max="7687" width="12.7265625" customWidth="1"/>
+    <col min="7688" max="7688" width="12.81640625" customWidth="1"/>
+    <col min="7689" max="7690" width="12.7265625" customWidth="1"/>
+    <col min="7691" max="7694" width="12.81640625" customWidth="1"/>
+    <col min="7695" max="7698" width="12.7265625" customWidth="1"/>
+    <col min="7937" max="7937" width="21.1796875" customWidth="1"/>
+    <col min="7938" max="7938" width="12.453125" customWidth="1"/>
+    <col min="7939" max="7943" width="12.7265625" customWidth="1"/>
+    <col min="7944" max="7944" width="12.81640625" customWidth="1"/>
+    <col min="7945" max="7946" width="12.7265625" customWidth="1"/>
+    <col min="7947" max="7950" width="12.81640625" customWidth="1"/>
+    <col min="7951" max="7954" width="12.7265625" customWidth="1"/>
+    <col min="8193" max="8193" width="21.1796875" customWidth="1"/>
+    <col min="8194" max="8194" width="12.453125" customWidth="1"/>
+    <col min="8195" max="8199" width="12.7265625" customWidth="1"/>
+    <col min="8200" max="8200" width="12.81640625" customWidth="1"/>
+    <col min="8201" max="8202" width="12.7265625" customWidth="1"/>
+    <col min="8203" max="8206" width="12.81640625" customWidth="1"/>
+    <col min="8207" max="8210" width="12.7265625" customWidth="1"/>
+    <col min="8449" max="8449" width="21.1796875" customWidth="1"/>
+    <col min="8450" max="8450" width="12.453125" customWidth="1"/>
+    <col min="8451" max="8455" width="12.7265625" customWidth="1"/>
+    <col min="8456" max="8456" width="12.81640625" customWidth="1"/>
+    <col min="8457" max="8458" width="12.7265625" customWidth="1"/>
+    <col min="8459" max="8462" width="12.81640625" customWidth="1"/>
+    <col min="8463" max="8466" width="12.7265625" customWidth="1"/>
+    <col min="8705" max="8705" width="21.1796875" customWidth="1"/>
+    <col min="8706" max="8706" width="12.453125" customWidth="1"/>
+    <col min="8707" max="8711" width="12.7265625" customWidth="1"/>
+    <col min="8712" max="8712" width="12.81640625" customWidth="1"/>
+    <col min="8713" max="8714" width="12.7265625" customWidth="1"/>
+    <col min="8715" max="8718" width="12.81640625" customWidth="1"/>
+    <col min="8719" max="8722" width="12.7265625" customWidth="1"/>
+    <col min="8961" max="8961" width="21.1796875" customWidth="1"/>
+    <col min="8962" max="8962" width="12.453125" customWidth="1"/>
+    <col min="8963" max="8967" width="12.7265625" customWidth="1"/>
+    <col min="8968" max="8968" width="12.81640625" customWidth="1"/>
+    <col min="8969" max="8970" width="12.7265625" customWidth="1"/>
+    <col min="8971" max="8974" width="12.81640625" customWidth="1"/>
+    <col min="8975" max="8978" width="12.7265625" customWidth="1"/>
+    <col min="9217" max="9217" width="21.1796875" customWidth="1"/>
+    <col min="9218" max="9218" width="12.453125" customWidth="1"/>
+    <col min="9219" max="9223" width="12.7265625" customWidth="1"/>
+    <col min="9224" max="9224" width="12.81640625" customWidth="1"/>
+    <col min="9225" max="9226" width="12.7265625" customWidth="1"/>
+    <col min="9227" max="9230" width="12.81640625" customWidth="1"/>
+    <col min="9231" max="9234" width="12.7265625" customWidth="1"/>
+    <col min="9473" max="9473" width="21.1796875" customWidth="1"/>
+    <col min="9474" max="9474" width="12.453125" customWidth="1"/>
+    <col min="9475" max="9479" width="12.7265625" customWidth="1"/>
+    <col min="9480" max="9480" width="12.81640625" customWidth="1"/>
+    <col min="9481" max="9482" width="12.7265625" customWidth="1"/>
+    <col min="9483" max="9486" width="12.81640625" customWidth="1"/>
+    <col min="9487" max="9490" width="12.7265625" customWidth="1"/>
+    <col min="9729" max="9729" width="21.1796875" customWidth="1"/>
+    <col min="9730" max="9730" width="12.453125" customWidth="1"/>
+    <col min="9731" max="9735" width="12.7265625" customWidth="1"/>
+    <col min="9736" max="9736" width="12.81640625" customWidth="1"/>
+    <col min="9737" max="9738" width="12.7265625" customWidth="1"/>
+    <col min="9739" max="9742" width="12.81640625" customWidth="1"/>
+    <col min="9743" max="9746" width="12.7265625" customWidth="1"/>
+    <col min="9985" max="9985" width="21.1796875" customWidth="1"/>
+    <col min="9986" max="9986" width="12.453125" customWidth="1"/>
+    <col min="9987" max="9991" width="12.7265625" customWidth="1"/>
+    <col min="9992" max="9992" width="12.81640625" customWidth="1"/>
+    <col min="9993" max="9994" width="12.7265625" customWidth="1"/>
+    <col min="9995" max="9998" width="12.81640625" customWidth="1"/>
+    <col min="9999" max="10002" width="12.7265625" customWidth="1"/>
+    <col min="10241" max="10241" width="21.1796875" customWidth="1"/>
+    <col min="10242" max="10242" width="12.453125" customWidth="1"/>
+    <col min="10243" max="10247" width="12.7265625" customWidth="1"/>
+    <col min="10248" max="10248" width="12.81640625" customWidth="1"/>
+    <col min="10249" max="10250" width="12.7265625" customWidth="1"/>
+    <col min="10251" max="10254" width="12.81640625" customWidth="1"/>
+    <col min="10255" max="10258" width="12.7265625" customWidth="1"/>
+    <col min="10497" max="10497" width="21.1796875" customWidth="1"/>
+    <col min="10498" max="10498" width="12.453125" customWidth="1"/>
+    <col min="10499" max="10503" width="12.7265625" customWidth="1"/>
+    <col min="10504" max="10504" width="12.81640625" customWidth="1"/>
+    <col min="10505" max="10506" width="12.7265625" customWidth="1"/>
+    <col min="10507" max="10510" width="12.81640625" customWidth="1"/>
+    <col min="10511" max="10514" width="12.7265625" customWidth="1"/>
+    <col min="10753" max="10753" width="21.1796875" customWidth="1"/>
+    <col min="10754" max="10754" width="12.453125" customWidth="1"/>
+    <col min="10755" max="10759" width="12.7265625" customWidth="1"/>
+    <col min="10760" max="10760" width="12.81640625" customWidth="1"/>
+    <col min="10761" max="10762" width="12.7265625" customWidth="1"/>
+    <col min="10763" max="10766" width="12.81640625" customWidth="1"/>
+    <col min="10767" max="10770" width="12.7265625" customWidth="1"/>
+    <col min="11009" max="11009" width="21.1796875" customWidth="1"/>
+    <col min="11010" max="11010" width="12.453125" customWidth="1"/>
+    <col min="11011" max="11015" width="12.7265625" customWidth="1"/>
+    <col min="11016" max="11016" width="12.81640625" customWidth="1"/>
+    <col min="11017" max="11018" width="12.7265625" customWidth="1"/>
+    <col min="11019" max="11022" width="12.81640625" customWidth="1"/>
+    <col min="11023" max="11026" width="12.7265625" customWidth="1"/>
+    <col min="11265" max="11265" width="21.1796875" customWidth="1"/>
+    <col min="11266" max="11266" width="12.453125" customWidth="1"/>
+    <col min="11267" max="11271" width="12.7265625" customWidth="1"/>
+    <col min="11272" max="11272" width="12.81640625" customWidth="1"/>
+    <col min="11273" max="11274" width="12.7265625" customWidth="1"/>
+    <col min="11275" max="11278" width="12.81640625" customWidth="1"/>
+    <col min="11279" max="11282" width="12.7265625" customWidth="1"/>
+    <col min="11521" max="11521" width="21.1796875" customWidth="1"/>
+    <col min="11522" max="11522" width="12.453125" customWidth="1"/>
+    <col min="11523" max="11527" width="12.7265625" customWidth="1"/>
+    <col min="11528" max="11528" width="12.81640625" customWidth="1"/>
+    <col min="11529" max="11530" width="12.7265625" customWidth="1"/>
+    <col min="11531" max="11534" width="12.81640625" customWidth="1"/>
+    <col min="11535" max="11538" width="12.7265625" customWidth="1"/>
+    <col min="11777" max="11777" width="21.1796875" customWidth="1"/>
+    <col min="11778" max="11778" width="12.453125" customWidth="1"/>
+    <col min="11779" max="11783" width="12.7265625" customWidth="1"/>
+    <col min="11784" max="11784" width="12.81640625" customWidth="1"/>
+    <col min="11785" max="11786" width="12.7265625" customWidth="1"/>
+    <col min="11787" max="11790" width="12.81640625" customWidth="1"/>
+    <col min="11791" max="11794" width="12.7265625" customWidth="1"/>
+    <col min="12033" max="12033" width="21.1796875" customWidth="1"/>
+    <col min="12034" max="12034" width="12.453125" customWidth="1"/>
+    <col min="12035" max="12039" width="12.7265625" customWidth="1"/>
+    <col min="12040" max="12040" width="12.81640625" customWidth="1"/>
+    <col min="12041" max="12042" width="12.7265625" customWidth="1"/>
+    <col min="12043" max="12046" width="12.81640625" customWidth="1"/>
+    <col min="12047" max="12050" width="12.7265625" customWidth="1"/>
+    <col min="12289" max="12289" width="21.1796875" customWidth="1"/>
+    <col min="12290" max="12290" width="12.453125" customWidth="1"/>
+    <col min="12291" max="12295" width="12.7265625" customWidth="1"/>
+    <col min="12296" max="12296" width="12.81640625" customWidth="1"/>
+    <col min="12297" max="12298" width="12.7265625" customWidth="1"/>
+    <col min="12299" max="12302" width="12.81640625" customWidth="1"/>
+    <col min="12303" max="12306" width="12.7265625" customWidth="1"/>
+    <col min="12545" max="12545" width="21.1796875" customWidth="1"/>
+    <col min="12546" max="12546" width="12.453125" customWidth="1"/>
+    <col min="12547" max="12551" width="12.7265625" customWidth="1"/>
+    <col min="12552" max="12552" width="12.81640625" customWidth="1"/>
+    <col min="12553" max="12554" width="12.7265625" customWidth="1"/>
+    <col min="12555" max="12558" width="12.81640625" customWidth="1"/>
+    <col min="12559" max="12562" width="12.7265625" customWidth="1"/>
+    <col min="12801" max="12801" width="21.1796875" customWidth="1"/>
+    <col min="12802" max="12802" width="12.453125" customWidth="1"/>
+    <col min="12803" max="12807" width="12.7265625" customWidth="1"/>
+    <col min="12808" max="12808" width="12.81640625" customWidth="1"/>
+    <col min="12809" max="12810" width="12.7265625" customWidth="1"/>
+    <col min="12811" max="12814" width="12.81640625" customWidth="1"/>
+    <col min="12815" max="12818" width="12.7265625" customWidth="1"/>
+    <col min="13057" max="13057" width="21.1796875" customWidth="1"/>
+    <col min="13058" max="13058" width="12.453125" customWidth="1"/>
+    <col min="13059" max="13063" width="12.7265625" customWidth="1"/>
+    <col min="13064" max="13064" width="12.81640625" customWidth="1"/>
+    <col min="13065" max="13066" width="12.7265625" customWidth="1"/>
+    <col min="13067" max="13070" width="12.81640625" customWidth="1"/>
+    <col min="13071" max="13074" width="12.7265625" customWidth="1"/>
+    <col min="13313" max="13313" width="21.1796875" customWidth="1"/>
+    <col min="13314" max="13314" width="12.453125" customWidth="1"/>
+    <col min="13315" max="13319" width="12.7265625" customWidth="1"/>
+    <col min="13320" max="13320" width="12.81640625" customWidth="1"/>
+    <col min="13321" max="13322" width="12.7265625" customWidth="1"/>
+    <col min="13323" max="13326" width="12.81640625" customWidth="1"/>
+    <col min="13327" max="13330" width="12.7265625" customWidth="1"/>
+    <col min="13569" max="13569" width="21.1796875" customWidth="1"/>
+    <col min="13570" max="13570" width="12.453125" customWidth="1"/>
+    <col min="13571" max="13575" width="12.7265625" customWidth="1"/>
+    <col min="13576" max="13576" width="12.81640625" customWidth="1"/>
+    <col min="13577" max="13578" width="12.7265625" customWidth="1"/>
+    <col min="13579" max="13582" width="12.81640625" customWidth="1"/>
+    <col min="13583" max="13586" width="12.7265625" customWidth="1"/>
+    <col min="13825" max="13825" width="21.1796875" customWidth="1"/>
+    <col min="13826" max="13826" width="12.453125" customWidth="1"/>
+    <col min="13827" max="13831" width="12.7265625" customWidth="1"/>
+    <col min="13832" max="13832" width="12.81640625" customWidth="1"/>
+    <col min="13833" max="13834" width="12.7265625" customWidth="1"/>
+    <col min="13835" max="13838" width="12.81640625" customWidth="1"/>
+    <col min="13839" max="13842" width="12.7265625" customWidth="1"/>
+    <col min="14081" max="14081" width="21.1796875" customWidth="1"/>
+    <col min="14082" max="14082" width="12.453125" customWidth="1"/>
+    <col min="14083" max="14087" width="12.7265625" customWidth="1"/>
+    <col min="14088" max="14088" width="12.81640625" customWidth="1"/>
+    <col min="14089" max="14090" width="12.7265625" customWidth="1"/>
+    <col min="14091" max="14094" width="12.81640625" customWidth="1"/>
+    <col min="14095" max="14098" width="12.7265625" customWidth="1"/>
+    <col min="14337" max="14337" width="21.1796875" customWidth="1"/>
+    <col min="14338" max="14338" width="12.453125" customWidth="1"/>
+    <col min="14339" max="14343" width="12.7265625" customWidth="1"/>
+    <col min="14344" max="14344" width="12.81640625" customWidth="1"/>
+    <col min="14345" max="14346" width="12.7265625" customWidth="1"/>
+    <col min="14347" max="14350" width="12.81640625" customWidth="1"/>
+    <col min="14351" max="14354" width="12.7265625" customWidth="1"/>
+    <col min="14593" max="14593" width="21.1796875" customWidth="1"/>
+    <col min="14594" max="14594" width="12.453125" customWidth="1"/>
+    <col min="14595" max="14599" width="12.7265625" customWidth="1"/>
+    <col min="14600" max="14600" width="12.81640625" customWidth="1"/>
+    <col min="14601" max="14602" width="12.7265625" customWidth="1"/>
+    <col min="14603" max="14606" width="12.81640625" customWidth="1"/>
+    <col min="14607" max="14610" width="12.7265625" customWidth="1"/>
+    <col min="14849" max="14849" width="21.1796875" customWidth="1"/>
+    <col min="14850" max="14850" width="12.453125" customWidth="1"/>
+    <col min="14851" max="14855" width="12.7265625" customWidth="1"/>
+    <col min="14856" max="14856" width="12.81640625" customWidth="1"/>
+    <col min="14857" max="14858" width="12.7265625" customWidth="1"/>
+    <col min="14859" max="14862" width="12.81640625" customWidth="1"/>
+    <col min="14863" max="14866" width="12.7265625" customWidth="1"/>
+    <col min="15105" max="15105" width="21.1796875" customWidth="1"/>
+    <col min="15106" max="15106" width="12.453125" customWidth="1"/>
+    <col min="15107" max="15111" width="12.7265625" customWidth="1"/>
+    <col min="15112" max="15112" width="12.81640625" customWidth="1"/>
+    <col min="15113" max="15114" width="12.7265625" customWidth="1"/>
+    <col min="15115" max="15118" width="12.81640625" customWidth="1"/>
+    <col min="15119" max="15122" width="12.7265625" customWidth="1"/>
+    <col min="15361" max="15361" width="21.1796875" customWidth="1"/>
+    <col min="15362" max="15362" width="12.453125" customWidth="1"/>
+    <col min="15363" max="15367" width="12.7265625" customWidth="1"/>
+    <col min="15368" max="15368" width="12.81640625" customWidth="1"/>
+    <col min="15369" max="15370" width="12.7265625" customWidth="1"/>
+    <col min="15371" max="15374" width="12.81640625" customWidth="1"/>
+    <col min="15375" max="15378" width="12.7265625" customWidth="1"/>
+    <col min="15617" max="15617" width="21.1796875" customWidth="1"/>
+    <col min="15618" max="15618" width="12.453125" customWidth="1"/>
+    <col min="15619" max="15623" width="12.7265625" customWidth="1"/>
+    <col min="15624" max="15624" width="12.81640625" customWidth="1"/>
+    <col min="15625" max="15626" width="12.7265625" customWidth="1"/>
+    <col min="15627" max="15630" width="12.81640625" customWidth="1"/>
+    <col min="15631" max="15634" width="12.7265625" customWidth="1"/>
+    <col min="15873" max="15873" width="21.1796875" customWidth="1"/>
+    <col min="15874" max="15874" width="12.453125" customWidth="1"/>
+    <col min="15875" max="15879" width="12.7265625" customWidth="1"/>
+    <col min="15880" max="15880" width="12.81640625" customWidth="1"/>
+    <col min="15881" max="15882" width="12.7265625" customWidth="1"/>
+    <col min="15883" max="15886" width="12.81640625" customWidth="1"/>
+    <col min="15887" max="15890" width="12.7265625" customWidth="1"/>
+    <col min="16129" max="16129" width="21.1796875" customWidth="1"/>
+    <col min="16130" max="16130" width="12.453125" customWidth="1"/>
+    <col min="16131" max="16135" width="12.7265625" customWidth="1"/>
+    <col min="16136" max="16136" width="12.81640625" customWidth="1"/>
+    <col min="16137" max="16138" width="12.7265625" customWidth="1"/>
+    <col min="16139" max="16142" width="12.81640625" customWidth="1"/>
+    <col min="16143" max="16146" width="12.7265625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:18">
@@ -18053,7 +18077,7 @@
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E4E8B5F8-CAC2-4F37-8597-58946AEA5DB1}">
   <dimension ref="A1:U25"/>
-  <sheetFormatPr defaultColWidth="19" defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="19" defaultRowHeight="14.5"/>
   <cols>
     <col min="1" max="1" width="19" customWidth="1"/>
   </cols>
@@ -19020,8 +19044,8 @@
         <v>44536.615934699075</v>
       </c>
     </row>
-    <row r="19" spans="1:21" ht="15.75" thickBot="1"/>
-    <row r="20" spans="1:21" ht="15.75" thickBot="1">
+    <row r="19" spans="1:21" ht="15" thickBot="1"/>
+    <row r="20" spans="1:21" ht="15" thickBot="1">
       <c r="A20" s="93"/>
       <c r="B20" s="94" t="s">
         <v>255</v>
@@ -19030,7 +19054,7 @@
         <v>256</v>
       </c>
     </row>
-    <row r="21" spans="1:21" ht="15.75" thickTop="1">
+    <row r="21" spans="1:21" ht="15" thickTop="1">
       <c r="A21" s="96" t="s">
         <v>252</v>
       </c>
@@ -19053,7 +19077,7 @@
         <v>0.48580480150021893</v>
       </c>
     </row>
-    <row r="23" spans="1:21" ht="15.75" thickBot="1">
+    <row r="23" spans="1:21" ht="15" thickBot="1">
       <c r="A23" s="69" t="s">
         <v>254</v>
       </c>
@@ -19226,18 +19250,18 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
   <Display>DocumentLibraryForm</Display>
   <Edit>DocumentLibraryForm</Edit>
   <New>DocumentLibraryForm</New>
 </FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -19259,18 +19283,18 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{30D49544-8BCC-440A-9096-15397E5D5534}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{63D16A6B-8B1B-4121-BE38-0F3E968A7BF0}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{30D49544-8BCC-440A-9096-15397E5D5534}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>